<commit_message>
Logica mejorada para el RIA 11 y 12
</commit_message>
<xml_diff>
--- a/data/dataset.xlsx
+++ b/data/dataset.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PIPRE-ML-IA\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\PIPRE-ML-IA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32D02C9-3A3B-43FA-A5C1-B56FD866690B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58655384-D13B-48A5-BDDC-2C34035C5092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -496,7 +501,18 @@
   <dimension ref="A1:S651"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="18" max="18" width="26.140625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
+    <col min="9" max="9" width="29" customWidth="1"/>
+    <col min="10" max="10" width="31.28515625" customWidth="1"/>
+    <col min="11" max="11" width="37" customWidth="1"/>
+    <col min="12" max="12" width="27.7109375" customWidth="1"/>
+    <col min="13" max="13" width="25.85546875" customWidth="1"/>
+    <col min="14" max="14" width="21.28515625" customWidth="1"/>
+    <col min="15" max="15" width="27.140625" customWidth="1"/>
+    <col min="16" max="16" width="30.140625" customWidth="1"/>
+    <col min="17" max="17" width="27.7109375" customWidth="1"/>
+    <col min="18" max="18" width="35.28515625" customWidth="1"/>
     <col min="19" max="19" width="20.85546875" customWidth="1"/>
     <col min="20" max="20" width="13.5703125" customWidth="1"/>
     <col min="21" max="21" width="25" customWidth="1"/>

</xml_diff>